<commit_message>
Sync generated repository state
</commit_message>
<xml_diff>
--- a/assets/downloads/sap-lead-assessment-master.xlsx
+++ b/assets/downloads/sap-lead-assessment-master.xlsx
@@ -147,7 +147,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9">
@@ -167,7 +167,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11">
@@ -188,7 +188,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">34.6%</t>
+          <t xml:space="preserve">34.8%</t>
         </is>
       </c>
     </row>
@@ -18468,42 +18468,42 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assessment Practice</t>
+          <t xml:space="preserve">Other / Cross-domain</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Labs — SAP Enterprise, Assurance, AI, Interview and Assessment</t>
+          <t xml:space="preserve">SAP Incident Diagnostics — Evidence to Incident Brief and RCA</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/</t>
+          <t xml:space="preserve">/labs/incident-diagnostics/</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/index.md</t>
+          <t xml:space="preserve">labs/incident-diagnostics/index.md</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_decision</t>
+          <t xml:space="preserve">mapped</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t xml:space="preserve">undeclared</t>
+          <t xml:space="preserve">mapped</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">integration-observability, integration-recovery, logistics-mdg</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-ams, delivery-memory, integration-cleancore</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -18521,7 +18521,7 @@
       </c>
       <c r="L225" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/incident-diagnostics/</t>
         </is>
       </c>
       <c r="M225" t="inlineStr">
@@ -18533,42 +18533,42 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interview Readiness</t>
+          <t xml:space="preserve">Assessment Practice</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Boss Battles — Long-form Interview Pressure Cases</t>
+          <t xml:space="preserve">Labs — SAP Enterprise, Assurance, AI, Interview and Assessment</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/boss-battles/</t>
+          <t xml:space="preserve">/labs/</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/interview-readiness/boss-battles/index.md</t>
+          <t xml:space="preserve">labs/index.md</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t xml:space="preserve">mapped</t>
+          <t xml:space="preserve">needs_decision</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t xml:space="preserve">mapped</t>
+          <t xml:space="preserve">undeclared</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-readiness, integration-ownership, lead-answer, lead-challenge, lead-decision, lead-stakeholders, logistics-p2p, sales-o2c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">delivery-ams, delivery-memory, integration-cleancore</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -18586,7 +18586,7 @@
       </c>
       <c r="L226" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/boss-battles/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/</t>
         </is>
       </c>
       <c r="M226" t="inlineStr">
@@ -18603,17 +18603,17 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Contrast Lab — Distinguish the Right Boundary</t>
+          <t xml:space="preserve">SAP Lead Boss Battles — Long-form Interview Pressure Cases</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/contrast/</t>
+          <t xml:space="preserve">/labs/interview-readiness/boss-battles/</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/interview-readiness/contrast/index.md</t>
+          <t xml:space="preserve">labs/interview-readiness/boss-battles/index.md</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
@@ -18628,7 +18628,7 @@
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-memory, delivery-testing, lead-answer</t>
+          <t xml:space="preserve">ai-readiness, integration-ownership, lead-answer, lead-challenge, lead-decision, lead-stakeholders, logistics-p2p, sales-o2c</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
@@ -18651,7 +18651,7 @@
       </c>
       <c r="L227" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/contrast/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/boss-battles/</t>
         </is>
       </c>
       <c r="M227" t="inlineStr">
@@ -18668,17 +18668,17 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Decision Cards — Architecture Trade-offs for Interviews</t>
+          <t xml:space="preserve">SAP Lead Contrast Lab — Distinguish the Right Boundary</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/decision-cards/</t>
+          <t xml:space="preserve">/labs/interview-readiness/contrast/</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/interview-readiness/decision-cards/index.md</t>
+          <t xml:space="preserve">labs/interview-readiness/contrast/index.md</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
@@ -18693,7 +18693,7 @@
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-readiness, integration-patterns, integration-recovery, lead-challenge, lead-decision, logistics-ewm</t>
+          <t xml:space="preserve">delivery-memory, delivery-testing, lead-answer</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
@@ -18716,7 +18716,7 @@
       </c>
       <c r="L228" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/decision-cards/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/contrast/</t>
         </is>
       </c>
       <c r="M228" t="inlineStr">
@@ -18733,17 +18733,17 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Diagnostic Lab — Production Failure Scenarios</t>
+          <t xml:space="preserve">SAP Lead Decision Cards — Architecture Trade-offs for Interviews</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/diagnostic-lab/</t>
+          <t xml:space="preserve">/labs/interview-readiness/decision-cards/</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/interview-readiness/diagnostic-lab/index.md</t>
+          <t xml:space="preserve">labs/interview-readiness/decision-cards/index.md</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
@@ -18758,7 +18758,7 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-testing, integration-recovery, logistics-inventory, sales-atp, sales-billing, sales-diagnostics</t>
+          <t xml:space="preserve">ai-readiness, integration-patterns, integration-recovery, lead-challenge, lead-decision, logistics-ewm</t>
         </is>
       </c>
       <c r="H229" t="inlineStr">
@@ -18781,7 +18781,7 @@
       </c>
       <c r="L229" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/diagnostic-lab/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/decision-cards/</t>
         </is>
       </c>
       <c r="M229" t="inlineStr">
@@ -18798,17 +18798,17 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Interview Drills — Decisions, Diagnostics, Pressure, Evidence</t>
+          <t xml:space="preserve">SAP Lead Diagnostic Lab — Production Failure Scenarios</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/drills/</t>
+          <t xml:space="preserve">/labs/interview-readiness/diagnostic-lab/</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/interview-readiness/drills/index.md</t>
+          <t xml:space="preserve">labs/interview-readiness/diagnostic-lab/index.md</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
@@ -18823,7 +18823,7 @@
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t xml:space="preserve">lead-answer, lead-challenge, lead-decision, lead-evidence</t>
+          <t xml:space="preserve">delivery-testing, integration-recovery, logistics-inventory, sales-atp, sales-billing, sales-diagnostics</t>
         </is>
       </c>
       <c r="H230" t="inlineStr">
@@ -18846,7 +18846,7 @@
       </c>
       <c r="L230" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/drills/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/diagnostic-lab/</t>
         </is>
       </c>
       <c r="M230" t="inlineStr">
@@ -18858,22 +18858,22 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t xml:space="preserve">AI / RAG / Agents</t>
+          <t xml:space="preserve">Interview Readiness</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Evidence Bank — Project Story Coverage</t>
+          <t xml:space="preserve">SAP Lead Interview Drills — Decisions, Diagnostics, Pressure, Evidence</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/evidence-bank/</t>
+          <t xml:space="preserve">/labs/interview-readiness/drills/</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/interview-readiness/evidence-bank/index.md</t>
+          <t xml:space="preserve">labs/interview-readiness/drills/index.md</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
@@ -18888,7 +18888,7 @@
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-ownership, lead-decision, lead-evidence, lead-stakeholders</t>
+          <t xml:space="preserve">lead-answer, lead-challenge, lead-decision, lead-evidence</t>
         </is>
       </c>
       <c r="H231" t="inlineStr">
@@ -18911,7 +18911,7 @@
       </c>
       <c r="L231" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/evidence-bank/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/drills/</t>
         </is>
       </c>
       <c r="M231" t="inlineStr">
@@ -18923,42 +18923,42 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interview Readiness</t>
+          <t xml:space="preserve">AI / RAG / Agents</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Interview Readiness — Practical Preparation Lab</t>
+          <t xml:space="preserve">SAP Lead Evidence Bank — Project Story Coverage</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/</t>
+          <t xml:space="preserve">/labs/interview-readiness/evidence-bank/</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/interview-readiness/index.md</t>
+          <t xml:space="preserve">labs/interview-readiness/evidence-bank/index.md</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_decision</t>
+          <t xml:space="preserve">mapped</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t xml:space="preserve">undeclared</t>
+          <t xml:space="preserve">mapped</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">integration-ownership, lead-decision, lead-evidence, lead-stakeholders</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-ams, logistics-tm, sales-shipping</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -18976,7 +18976,7 @@
       </c>
       <c r="L232" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/evidence-bank/</t>
         </is>
       </c>
       <c r="M232" t="inlineStr">
@@ -18993,37 +18993,37 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Learning Science — Evidence Learning Engine</t>
+          <t xml:space="preserve">SAP Lead Interview Readiness — Practical Preparation Lab</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/learning-science/</t>
+          <t xml:space="preserve">/labs/interview-readiness/</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/interview-readiness/learning-science/index.md</t>
+          <t xml:space="preserve">labs/interview-readiness/index.md</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t xml:space="preserve">mapped</t>
+          <t xml:space="preserve">needs_decision</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t xml:space="preserve">mapped</t>
+          <t xml:space="preserve">undeclared</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-memory, delivery-testing, lead-answer</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">delivery-ams, logistics-tm, sales-shipping</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
@@ -19041,7 +19041,7 @@
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/learning-science/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/</t>
         </is>
       </c>
       <c r="M233" t="inlineStr">
@@ -19058,17 +19058,17 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Memory Atlas — Rebuild O2C, P2P and Integration</t>
+          <t xml:space="preserve">SAP Lead Learning Science — Evidence Learning Engine</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/memory-atlas/</t>
+          <t xml:space="preserve">/labs/interview-readiness/learning-science/</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/interview-readiness/memory-atlas/index.md</t>
+          <t xml:space="preserve">labs/interview-readiness/learning-science/index.md</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
@@ -19083,7 +19083,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-patterns, integration-recovery, logistics-p2p, sales-o2c</t>
+          <t xml:space="preserve">delivery-memory, delivery-testing, lead-answer</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
@@ -19106,7 +19106,7 @@
       </c>
       <c r="L234" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/memory-atlas/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/learning-science/</t>
         </is>
       </c>
       <c r="M234" t="inlineStr">
@@ -19123,37 +19123,37 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Interview Practice — 12-Question Interview Mode</t>
+          <t xml:space="preserve">SAP Lead Memory Atlas — Rebuild O2C, P2P and Integration</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/practice/</t>
+          <t xml:space="preserve">/labs/interview-readiness/memory-atlas/</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/interview-readiness/practice/index.md</t>
+          <t xml:space="preserve">labs/interview-readiness/memory-atlas/index.md</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_decision</t>
+          <t xml:space="preserve">mapped</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t xml:space="preserve">undeclared</t>
+          <t xml:space="preserve">mapped</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">integration-patterns, integration-recovery, logistics-p2p, sales-o2c</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-ams, logistics-tm, delivery-lifecycle</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -19171,7 +19171,7 @@
       </c>
       <c r="L235" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/practice/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/memory-atlas/</t>
         </is>
       </c>
       <c r="M235" t="inlineStr">
@@ -19188,17 +19188,17 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Interview Progress — Readiness and Weak Areas</t>
+          <t xml:space="preserve">SAP Lead Interview Practice — 12-Question Interview Mode</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/progress/</t>
+          <t xml:space="preserve">/labs/interview-readiness/practice/</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/interview-readiness/progress/index.md</t>
+          <t xml:space="preserve">labs/interview-readiness/practice/index.md</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
@@ -19218,7 +19218,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t xml:space="preserve">lead-evidence, ai-readiness, delivery-testing</t>
+          <t xml:space="preserve">delivery-ams, logistics-tm, delivery-lifecycle</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -19236,7 +19236,7 @@
       </c>
       <c r="L236" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/progress/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/practice/</t>
         </is>
       </c>
       <c r="M236" t="inlineStr">
@@ -19253,17 +19253,17 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Interview Questions — 42 Skills, 168 Questions</t>
+          <t xml:space="preserve">SAP Lead Interview Progress — Readiness and Weak Areas</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/questions/</t>
+          <t xml:space="preserve">/labs/interview-readiness/progress/</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/interview-readiness/questions/index.md</t>
+          <t xml:space="preserve">labs/interview-readiness/progress/index.md</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
@@ -19283,7 +19283,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-tm, delivery-ams, integration-ownership</t>
+          <t xml:space="preserve">lead-evidence, ai-readiness, delivery-testing</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
@@ -19301,7 +19301,7 @@
       </c>
       <c r="L237" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/questions/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/progress/</t>
         </is>
       </c>
       <c r="M237" t="inlineStr">
@@ -19318,17 +19318,17 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Career Roadmap — Skills, Labs, Evidence, Practice</t>
+          <t xml:space="preserve">SAP Lead Interview Questions — 42 Skills, 168 Questions</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/roadmap/</t>
+          <t xml:space="preserve">/labs/interview-readiness/questions/</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/interview-readiness/roadmap/index.md</t>
+          <t xml:space="preserve">labs/interview-readiness/questions/index.md</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
@@ -19348,7 +19348,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-ams, logistics-tm, delivery-lifecycle</t>
+          <t xml:space="preserve">logistics-tm, delivery-ams, integration-ownership</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
@@ -19366,7 +19366,7 @@
       </c>
       <c r="L238" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/roadmap/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/questions/</t>
         </is>
       </c>
       <c r="M238" t="inlineStr">
@@ -19383,17 +19383,17 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Interview Story Bank — Projects, Decisions, Failures, Results</t>
+          <t xml:space="preserve">SAP Lead Career Roadmap — Skills, Labs, Evidence, Practice</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/stories/</t>
+          <t xml:space="preserve">/labs/interview-readiness/roadmap/</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/interview-readiness/stories/index.md</t>
+          <t xml:space="preserve">labs/interview-readiness/roadmap/index.md</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
@@ -19413,7 +19413,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t xml:space="preserve">lead-evidence, integration-deployment, ai-agents-mcp</t>
+          <t xml:space="preserve">delivery-ams, logistics-tm, delivery-lifecycle</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -19431,7 +19431,7 @@
       </c>
       <c r="L239" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/stories/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/roadmap/</t>
         </is>
       </c>
       <c r="M239" t="inlineStr">
@@ -19448,37 +19448,37 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Mastery Today — Recall, Apply, Retain</t>
+          <t xml:space="preserve">SAP Interview Story Bank — Projects, Decisions, Failures, Results</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/today/</t>
+          <t xml:space="preserve">/labs/interview-readiness/stories/</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/interview-readiness/today/index.md</t>
+          <t xml:space="preserve">labs/interview-readiness/stories/index.md</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t xml:space="preserve">mapped</t>
+          <t xml:space="preserve">needs_decision</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t xml:space="preserve">mapped</t>
+          <t xml:space="preserve">undeclared</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-memory, delivery-testing, lead-answer</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">lead-evidence, integration-deployment, ai-agents-mcp</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
@@ -19496,7 +19496,7 @@
       </c>
       <c r="L240" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/today/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/stories/</t>
         </is>
       </c>
       <c r="M240" t="inlineStr">
@@ -19508,37 +19508,37 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reusable Data Procedures</t>
+          <t xml:space="preserve">Interview Readiness</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reusable Data Procedures</t>
+          <t xml:space="preserve">SAP Lead Mastery Today — Recall, Apply, Retain</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/reusable-data-procedures/</t>
+          <t xml:space="preserve">/labs/interview-readiness/today/</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/reusable-data-procedures/index.html</t>
+          <t xml:space="preserve">labs/interview-readiness/today/index.md</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_decision</t>
+          <t xml:space="preserve">mapped</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t xml:space="preserve">undeclared</t>
+          <t xml:space="preserve">mapped</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">delivery-memory, delivery-testing, lead-answer</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
@@ -19548,7 +19548,7 @@
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="J241" t="n">
@@ -19561,7 +19561,7 @@
       </c>
       <c r="L241" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/reusable-data-procedures/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/today/</t>
         </is>
       </c>
       <c r="M241" t="inlineStr">
@@ -19573,27 +19573,27 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t xml:space="preserve">Templates / Work Artifacts</t>
+          <t xml:space="preserve">Reusable Data Procedures</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operational Templates — RCA and Procedures</t>
+          <t xml:space="preserve">Reusable Data Procedures</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/templates/</t>
+          <t xml:space="preserve">/labs/reusable-data-procedures/</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/templates/index.md</t>
+          <t xml:space="preserve">labs/reusable-data-procedures/index.html</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t xml:space="preserve">mapped</t>
+          <t xml:space="preserve">needs_decision</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
@@ -19603,7 +19603,7 @@
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-memory</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H242" t="inlineStr">
@@ -19613,7 +19613,7 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t xml:space="preserve">P3</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="J242" t="n">
@@ -19626,7 +19626,7 @@
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/templates/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/reusable-data-procedures/</t>
         </is>
       </c>
       <c r="M242" t="inlineStr">
@@ -19638,37 +19638,37 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assessment Practice</t>
+          <t xml:space="preserve">Templates / Work Artifacts</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Assessment Master Workbook</t>
+          <t xml:space="preserve">Operational Templates — RCA and Procedures</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/templates/sap-lead-assessment-prep/</t>
+          <t xml:space="preserve">/labs/templates/</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t xml:space="preserve">labs/templates/sap-lead-assessment-prep.md</t>
+          <t xml:space="preserve">labs/templates/index.md</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t xml:space="preserve">excluded</t>
+          <t xml:space="preserve">mapped</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t xml:space="preserve">none</t>
+          <t xml:space="preserve">undeclared</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">delivery-memory</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
@@ -19691,7 +19691,7 @@
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/templates/sap-lead-assessment-prep/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/templates/</t>
         </is>
       </c>
       <c r="M243" t="inlineStr">
@@ -19703,70 +19703,135 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
+          <t xml:space="preserve">Assessment Practice</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAP Lead Assessment Master Workbook</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/labs/templates/sap-lead-assessment-prep/</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">labs/templates/sap-lead-assessment-prep.md</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">excluded</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">none</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P3</t>
+        </is>
+      </c>
+      <c r="J244" t="n">
+        <v>1</v>
+      </c>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/templates/sap-lead-assessment-prep/</t>
+        </is>
+      </c>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
           <t xml:space="preserve">Tooling / Roadmap</t>
         </is>
       </c>
-      <c r="B244" t="inlineStr">
+      <c r="B245" t="inlineStr">
         <is>
           <t xml:space="preserve">Tool Roadmap — Portable Enterprise Tools</t>
         </is>
       </c>
-      <c r="C244" t="inlineStr">
+      <c r="C245" t="inlineStr">
         <is>
           <t xml:space="preserve">/labs/tool-roadmap/</t>
         </is>
       </c>
-      <c r="D244" t="inlineStr">
+      <c r="D245" t="inlineStr">
         <is>
           <t xml:space="preserve">labs/tool-roadmap/index.md</t>
         </is>
       </c>
-      <c r="E244" t="inlineStr">
+      <c r="E245" t="inlineStr">
         <is>
           <t xml:space="preserve">needs_decision</t>
         </is>
       </c>
-      <c r="F244" t="inlineStr">
+      <c r="F245" t="inlineStr">
         <is>
           <t xml:space="preserve">undeclared</t>
         </is>
       </c>
-      <c r="G244" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H244" t="inlineStr">
+      <c r="G245" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
         <is>
           <t xml:space="preserve">delivery-testing, ai-agents-mcp, ai-data-governance</t>
         </is>
       </c>
-      <c r="I244" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="J244" t="n">
-        <v>1</v>
-      </c>
-      <c r="K244" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not Started</t>
-        </is>
-      </c>
-      <c r="L244" t="inlineStr">
+      <c r="I245" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="J245" t="n">
+        <v>1</v>
+      </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="L245" t="inlineStr">
         <is>
           <t xml:space="preserve">https://dkharlanau.github.io/labs/tool-roadmap/</t>
         </is>
       </c>
-      <c r="M244" t="inlineStr">
+      <c r="M245" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M244"/>
+  <autoFilter ref="A1:M245"/>
 </worksheet>
 </file>
 
@@ -20552,10 +20617,10 @@
         <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E35" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F35" t="n">
         <v>21</v>

</xml_diff>